<commit_message>
Add tests for user defined date
</commit_message>
<xml_diff>
--- a/TestComponents/TestSets/CropStage/FieldConfigs.xlsx
+++ b/TestComponents/TestSets/CropStage/FieldConfigs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubRepos\FieldNBalance\TestComponents\TestSets\CropStage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8828BC79-DAA0-4B46-A108-7DC510919ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{529D3AD6-94E2-444D-A141-F3AF157A1609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D0D9F3F3-C1B3-4B79-AF5D-93A117BC34BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D0D9F3F3-C1B3-4B79-AF5D-93A117BC34BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="72">
   <si>
     <t>InitialN</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t>Top30cm</t>
+  </si>
+  <si>
+    <t>FinalFertDate</t>
   </si>
 </sst>
 </file>
@@ -650,14 +653,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B67FC6C2-7F6C-4E8B-9465-EDB17589DEC5}">
-  <dimension ref="A1:O47"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="27.33203125" customWidth="1"/>
-    <col min="3" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
+    <col min="3" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>62</v>
       </c>
@@ -698,7 +701,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
         <v>17</v>
       </c>
@@ -739,7 +742,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:15" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>48</v>
       </c>
@@ -795,7 +798,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>49</v>
       </c>
@@ -854,7 +857,7 @@
         <v>lincoln</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" t="s">
         <v>0</v>
@@ -863,7 +866,7 @@
         <v>500</v>
       </c>
       <c r="D5">
-        <f t="shared" ref="D5:H47" si="8">C5</f>
+        <f t="shared" ref="D5:H48" si="8">C5</f>
         <v>500</v>
       </c>
       <c r="E5">
@@ -911,7 +914,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" t="s">
         <v>56</v>
@@ -968,7 +971,7 @@
         <v>Sedimentary</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" t="s">
         <v>58</v>
@@ -1025,7 +1028,7 @@
         <v>Silt</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" t="s">
         <v>59</v>
@@ -1082,7 +1085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" t="s">
         <v>1</v>
@@ -1127,7 +1130,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" t="s">
         <v>2</v>
@@ -1184,7 +1187,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" t="s">
         <v>3</v>
@@ -1241,7 +1244,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" t="s">
         <v>4</v>
@@ -1298,7 +1301,7 @@
         <v>Typical</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" t="s">
         <v>6</v>
@@ -1355,240 +1358,189 @@
         <v>Very Dry</v>
       </c>
     </row>
-    <row r="14" spans="1:15" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="8"/>
+      <c r="B15" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="1" t="str">
+      <c r="D15" s="1" t="str">
         <f t="shared" si="8"/>
         <v>Full</v>
       </c>
-      <c r="E14" s="1" t="str">
+      <c r="E15" s="1" t="str">
         <f t="shared" si="8"/>
         <v>Full</v>
       </c>
-      <c r="F14" s="1" t="str">
+      <c r="F15" s="1" t="str">
         <f t="shared" si="8"/>
         <v>Full</v>
       </c>
-      <c r="G14" s="1" t="str">
+      <c r="G15" s="1" t="str">
         <f t="shared" si="8"/>
         <v>Full</v>
       </c>
-      <c r="H14" s="1" t="str">
+      <c r="H15" s="1" t="str">
         <f t="shared" si="8"/>
         <v>Full</v>
       </c>
-      <c r="I14" s="1" t="str">
-        <f t="shared" ref="I14:O14" si="17">H14</f>
+      <c r="I15" s="1" t="str">
+        <f t="shared" ref="I15:O15" si="17">H15</f>
         <v>Full</v>
       </c>
-      <c r="J14" s="1" t="str">
+      <c r="J15" s="1" t="str">
         <f t="shared" si="17"/>
         <v>Full</v>
       </c>
-      <c r="K14" s="1" t="str">
+      <c r="K15" s="1" t="str">
         <f t="shared" si="17"/>
         <v>Full</v>
       </c>
-      <c r="L14" s="1" t="str">
+      <c r="L15" s="1" t="str">
         <f t="shared" si="17"/>
         <v>Full</v>
       </c>
-      <c r="M14" s="1" t="str">
+      <c r="M15" s="1" t="str">
         <f t="shared" si="17"/>
         <v>Full</v>
       </c>
-      <c r="N14" s="1" t="str">
+      <c r="N15" s="1" t="str">
         <f t="shared" si="17"/>
         <v>Full</v>
       </c>
-      <c r="O14" s="1" t="str">
+      <c r="O15" s="1" t="str">
         <f t="shared" si="17"/>
         <v>Full</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>10</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" t="s">
         <v>11</v>
       </c>
-      <c r="D15" t="str">
+      <c r="D16" t="str">
         <f t="shared" si="8"/>
         <v>TestResidue05</v>
       </c>
-      <c r="E15" t="str">
+      <c r="E16" t="str">
         <f t="shared" si="8"/>
         <v>TestResidue05</v>
       </c>
-      <c r="F15" t="str">
+      <c r="F16" t="str">
         <f t="shared" si="8"/>
         <v>TestResidue05</v>
       </c>
-      <c r="G15" t="str">
+      <c r="G16" t="str">
         <f t="shared" si="8"/>
         <v>TestResidue05</v>
       </c>
-      <c r="H15" t="str">
+      <c r="H16" t="str">
         <f t="shared" si="8"/>
         <v>TestResidue05</v>
       </c>
-      <c r="I15" t="str">
-        <f t="shared" ref="I15:O15" si="18">H15</f>
+      <c r="I16" t="str">
+        <f t="shared" ref="I16:O16" si="18">H16</f>
         <v>TestResidue05</v>
       </c>
-      <c r="J15" t="str">
+      <c r="J16" t="str">
         <f t="shared" si="18"/>
         <v>TestResidue05</v>
       </c>
-      <c r="K15" t="str">
+      <c r="K16" t="str">
         <f t="shared" si="18"/>
         <v>TestResidue05</v>
       </c>
-      <c r="L15" t="str">
+      <c r="L16" t="str">
         <f t="shared" si="18"/>
         <v>TestResidue05</v>
       </c>
-      <c r="M15" t="str">
+      <c r="M16" t="str">
         <f t="shared" si="18"/>
         <v>TestResidue05</v>
       </c>
-      <c r="N15" t="str">
+      <c r="N16" t="str">
         <f t="shared" si="18"/>
         <v>TestResidue05</v>
       </c>
-      <c r="O15" t="str">
+      <c r="O16" t="str">
         <f t="shared" si="18"/>
         <v>TestResidue05</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" t="s">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" t="s">
         <v>53</v>
       </c>
-      <c r="C16">
+      <c r="C17">
         <v>13</v>
       </c>
-      <c r="D16">
+      <c r="D17">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="E16">
+      <c r="E17">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="F16">
+      <c r="F17">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="G16">
+      <c r="G17">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="H16">
+      <c r="H17">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="I16">
-        <f t="shared" ref="I16:O16" si="19">H16</f>
+      <c r="I17">
+        <f t="shared" ref="I17:O17" si="19">H17</f>
         <v>13</v>
       </c>
-      <c r="J16">
+      <c r="J17">
         <f t="shared" si="19"/>
         <v>13</v>
       </c>
-      <c r="K16">
+      <c r="K17">
         <f t="shared" si="19"/>
         <v>13</v>
       </c>
-      <c r="L16">
+      <c r="L17">
         <f t="shared" si="19"/>
         <v>13</v>
       </c>
-      <c r="M16">
+      <c r="M17">
         <f t="shared" si="19"/>
         <v>13</v>
       </c>
-      <c r="N16">
+      <c r="N17">
         <f t="shared" si="19"/>
         <v>13</v>
       </c>
-      <c r="O16">
+      <c r="O17">
         <f t="shared" si="19"/>
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A17" s="9"/>
-      <c r="B17" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="G17">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="H17">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="I17">
-        <f t="shared" ref="I17:O17" si="20">H17</f>
-        <v>0</v>
-      </c>
-      <c r="J17">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="K17">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="M17">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="N17">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="O17">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="9"/>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -1614,609 +1566,609 @@
         <v>0</v>
       </c>
       <c r="I18">
-        <f t="shared" ref="I18:O18" si="21">H18</f>
+        <f t="shared" ref="I18:O18" si="20">H18</f>
         <v>0</v>
       </c>
       <c r="J18">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="K18">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="L18">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="M18">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="N18">
-        <f t="shared" si="21"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="O18">
-        <f t="shared" si="21"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="9"/>
       <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <f t="shared" ref="I19:O19" si="21">H19</f>
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="9"/>
+      <c r="B20" t="s">
         <v>14</v>
       </c>
-      <c r="C19">
+      <c r="C20">
         <v>13</v>
       </c>
-      <c r="D19">
+      <c r="D20">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="E19">
+      <c r="E20">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="F19">
+      <c r="F20">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="G19">
+      <c r="G20">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="H19">
+      <c r="H20">
         <f t="shared" si="8"/>
         <v>13</v>
       </c>
-      <c r="I19">
-        <f t="shared" ref="I19:O19" si="22">H19</f>
+      <c r="I20">
+        <f t="shared" ref="I20:O20" si="22">H20</f>
         <v>13</v>
       </c>
-      <c r="J19">
+      <c r="J20">
         <f t="shared" si="22"/>
         <v>13</v>
       </c>
-      <c r="K19">
+      <c r="K20">
         <f t="shared" si="22"/>
         <v>13</v>
       </c>
-      <c r="L19">
+      <c r="L20">
         <f t="shared" si="22"/>
         <v>13</v>
       </c>
-      <c r="M19">
+      <c r="M20">
         <f t="shared" si="22"/>
         <v>13</v>
       </c>
-      <c r="N19">
+      <c r="N20">
         <f t="shared" si="22"/>
         <v>13</v>
       </c>
-      <c r="O19">
+      <c r="O20">
         <f t="shared" si="22"/>
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="9"/>
-      <c r="B20" t="s">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="9"/>
+      <c r="B21" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C21" s="4">
         <v>44831</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D21" s="4">
         <f t="shared" si="8"/>
         <v>44831</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E21" s="4">
         <f t="shared" si="8"/>
         <v>44831</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F21" s="4">
         <f t="shared" si="8"/>
         <v>44831</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G21" s="4">
         <f t="shared" si="8"/>
         <v>44831</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H21" s="4">
         <f t="shared" si="8"/>
         <v>44831</v>
       </c>
-      <c r="I20" s="4">
-        <f t="shared" ref="I20:O20" si="23">H20</f>
+      <c r="I21" s="4">
+        <f t="shared" ref="I21:O21" si="23">H21</f>
         <v>44831</v>
       </c>
-      <c r="J20" s="4">
+      <c r="J21" s="4">
         <f t="shared" si="23"/>
         <v>44831</v>
       </c>
-      <c r="K20" s="4">
+      <c r="K21" s="4">
         <f t="shared" si="23"/>
         <v>44831</v>
       </c>
-      <c r="L20" s="4">
+      <c r="L21" s="4">
         <f t="shared" si="23"/>
         <v>44831</v>
       </c>
-      <c r="M20" s="4">
+      <c r="M21" s="4">
         <f t="shared" si="23"/>
         <v>44831</v>
       </c>
-      <c r="N20" s="4">
+      <c r="N21" s="4">
         <f t="shared" si="23"/>
         <v>44831</v>
       </c>
-      <c r="O20" s="4">
+      <c r="O21" s="4">
         <f t="shared" si="23"/>
         <v>44831</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="9"/>
-      <c r="B21" t="s">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
+      <c r="B22" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="3" t="str">
+      <c r="D22" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="E21" s="3" t="str">
+      <c r="E22" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="F21" s="3" t="str">
+      <c r="F22" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="G21" s="3" t="str">
+      <c r="G22" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="H21" s="3" t="str">
+      <c r="H22" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="I21" s="3" t="str">
-        <f t="shared" ref="I21:O21" si="24">H21</f>
+      <c r="I22" s="3" t="str">
+        <f t="shared" ref="I22:O22" si="24">H22</f>
         <v>Seed</v>
       </c>
-      <c r="J21" s="3" t="str">
+      <c r="J22" s="3" t="str">
         <f t="shared" si="24"/>
         <v>Seed</v>
       </c>
-      <c r="K21" s="3" t="str">
+      <c r="K22" s="3" t="str">
         <f t="shared" si="24"/>
         <v>Seed</v>
       </c>
-      <c r="L21" s="3" t="str">
+      <c r="L22" s="3" t="str">
         <f t="shared" si="24"/>
         <v>Seed</v>
       </c>
-      <c r="M21" s="3" t="str">
+      <c r="M22" s="3" t="str">
         <f t="shared" si="24"/>
         <v>Seed</v>
       </c>
-      <c r="N21" s="3" t="str">
+      <c r="N22" s="3" t="str">
         <f t="shared" si="24"/>
         <v>Seed</v>
       </c>
-      <c r="O21" s="3" t="str">
+      <c r="O22" s="3" t="str">
         <f t="shared" si="24"/>
         <v>Seed</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A22" s="9"/>
-      <c r="B22" t="s">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="9"/>
+      <c r="B23" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C23" s="4">
         <v>45010</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D23" s="4">
         <f t="shared" si="8"/>
         <v>45010</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E23" s="4">
         <f t="shared" si="8"/>
         <v>45010</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F23" s="4">
         <f t="shared" si="8"/>
         <v>45010</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G23" s="4">
         <f t="shared" si="8"/>
         <v>45010</v>
       </c>
-      <c r="H22" s="4">
+      <c r="H23" s="4">
         <f t="shared" si="8"/>
         <v>45010</v>
       </c>
-      <c r="I22" s="4">
-        <f t="shared" ref="I22:O22" si="25">H22</f>
+      <c r="I23" s="4">
+        <f t="shared" ref="I23:O23" si="25">H23</f>
         <v>45010</v>
       </c>
-      <c r="J22" s="4">
+      <c r="J23" s="4">
         <f t="shared" si="25"/>
         <v>45010</v>
       </c>
-      <c r="K22" s="4">
+      <c r="K23" s="4">
         <f t="shared" si="25"/>
         <v>45010</v>
       </c>
-      <c r="L22" s="4">
+      <c r="L23" s="4">
         <f t="shared" si="25"/>
         <v>45010</v>
       </c>
-      <c r="M22" s="4">
+      <c r="M23" s="4">
         <f t="shared" si="25"/>
         <v>45010</v>
       </c>
-      <c r="N22" s="4">
+      <c r="N23" s="4">
         <f t="shared" si="25"/>
         <v>45010</v>
       </c>
-      <c r="O22" s="4">
+      <c r="O23" s="4">
         <f t="shared" si="25"/>
         <v>45010</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A23" s="9"/>
-      <c r="B23" t="s">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="3" t="str">
+      <c r="D24" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Maturity</v>
       </c>
-      <c r="E23" s="3" t="str">
+      <c r="E24" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Maturity</v>
       </c>
-      <c r="F23" s="3" t="str">
+      <c r="F24" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Maturity</v>
       </c>
-      <c r="G23" s="3" t="str">
+      <c r="G24" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Maturity</v>
       </c>
-      <c r="H23" s="3" t="str">
+      <c r="H24" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Maturity</v>
       </c>
-      <c r="I23" s="3" t="str">
-        <f t="shared" ref="I23:O23" si="26">H23</f>
+      <c r="I24" s="3" t="str">
+        <f t="shared" ref="I24:O24" si="26">H24</f>
         <v>Maturity</v>
       </c>
-      <c r="J23" s="3" t="str">
+      <c r="J24" s="3" t="str">
         <f t="shared" si="26"/>
         <v>Maturity</v>
       </c>
-      <c r="K23" s="3" t="str">
+      <c r="K24" s="3" t="str">
         <f t="shared" si="26"/>
         <v>Maturity</v>
       </c>
-      <c r="L23" s="3" t="str">
+      <c r="L24" s="3" t="str">
         <f t="shared" si="26"/>
         <v>Maturity</v>
       </c>
-      <c r="M23" s="3" t="str">
+      <c r="M24" s="3" t="str">
         <f t="shared" si="26"/>
         <v>Maturity</v>
       </c>
-      <c r="N23" s="3" t="str">
+      <c r="N24" s="3" t="str">
         <f t="shared" si="26"/>
         <v>Maturity</v>
       </c>
-      <c r="O23" s="3" t="str">
+      <c r="O24" s="3" t="str">
         <f t="shared" si="26"/>
         <v>Maturity</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A24" s="9"/>
-      <c r="B24" t="s">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="9"/>
+      <c r="B25" t="s">
         <v>21</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C25" t="s">
         <v>22</v>
       </c>
-      <c r="D24" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="E24" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="F24" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="G24" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="H24" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="I24" t="str">
-        <f t="shared" ref="I24:O24" si="27">H24</f>
-        <v>None removed</v>
-      </c>
-      <c r="J24" t="str">
+      <c r="D25" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="F25" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="G25" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="H25" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="I25" t="str">
+        <f t="shared" ref="I25:O25" si="27">H25</f>
+        <v>None removed</v>
+      </c>
+      <c r="J25" t="str">
         <f t="shared" si="27"/>
         <v>None removed</v>
       </c>
-      <c r="K24" t="str">
+      <c r="K25" t="str">
         <f t="shared" si="27"/>
         <v>None removed</v>
       </c>
-      <c r="L24" t="str">
+      <c r="L25" t="str">
         <f t="shared" si="27"/>
         <v>None removed</v>
       </c>
-      <c r="M24" t="str">
+      <c r="M25" t="str">
         <f t="shared" si="27"/>
         <v>None removed</v>
       </c>
-      <c r="N24" t="str">
+      <c r="N25" t="str">
         <f t="shared" si="27"/>
         <v>None removed</v>
       </c>
-      <c r="O24" t="str">
+      <c r="O25" t="str">
         <f t="shared" si="27"/>
         <v>None removed</v>
       </c>
     </row>
-    <row r="25" spans="1:15" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="9"/>
-      <c r="B25" s="1" t="s">
+    <row r="26" spans="1:15" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="9"/>
+      <c r="B26" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="E25" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="F25" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="G25" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="H25" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="I25" s="1" t="str">
-        <f t="shared" ref="I25:O25" si="28">H25</f>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="J25" s="1" t="str">
+      <c r="D26" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="E26" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="F26" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="G26" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="H26" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="I26" s="1" t="str">
+        <f t="shared" ref="I26:O26" si="28">H26</f>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="J26" s="1" t="str">
         <f t="shared" si="28"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="K25" s="1" t="str">
+      <c r="K26" s="1" t="str">
         <f t="shared" si="28"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="L25" s="1" t="str">
+      <c r="L26" s="1" t="str">
         <f t="shared" si="28"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="M25" s="1" t="str">
+      <c r="M26" s="1" t="str">
         <f t="shared" si="28"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="N25" s="1" t="str">
+      <c r="N26" s="1" t="str">
         <f t="shared" si="28"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="O25" s="1" t="str">
+      <c r="O26" s="1" t="str">
         <f t="shared" si="28"/>
         <v>Full (Plough)</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>25</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C27" t="s">
         <v>61</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D27" t="str">
         <f t="shared" si="8"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="E26" t="str">
+      <c r="E27" t="str">
         <f t="shared" si="8"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="F26" t="str">
+      <c r="F27" t="str">
         <f t="shared" si="8"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="G26" t="str">
+      <c r="G27" t="str">
         <f t="shared" si="8"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="H26" t="str">
+      <c r="H27" t="str">
         <f t="shared" si="8"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="I26" t="str">
-        <f t="shared" ref="I26:N26" si="29">H26</f>
+      <c r="I27" t="str">
+        <f t="shared" ref="I27:N27" si="29">H27</f>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="J26" t="str">
+      <c r="J27" t="str">
         <f t="shared" si="29"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="K26" t="str">
+      <c r="K27" t="str">
         <f t="shared" si="29"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="L26" t="str">
+      <c r="L27" t="str">
         <f t="shared" si="29"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="M26" t="str">
+      <c r="M27" t="str">
         <f t="shared" si="29"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="N26" t="str">
+      <c r="N27" t="str">
         <f t="shared" si="29"/>
         <v>Wheat Grain Feed</v>
       </c>
-      <c r="O26" s="7" t="s">
+      <c r="O27" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A27" s="8"/>
-      <c r="B27" t="s">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" s="8"/>
+      <c r="B28" t="s">
         <v>54</v>
       </c>
-      <c r="C27">
+      <c r="C28">
         <v>10</v>
       </c>
-      <c r="D27">
+      <c r="D28">
         <f t="shared" si="8"/>
         <v>10</v>
       </c>
-      <c r="E27">
+      <c r="E28">
         <f t="shared" si="8"/>
         <v>10</v>
       </c>
-      <c r="F27">
+      <c r="F28">
         <f t="shared" si="8"/>
         <v>10</v>
       </c>
-      <c r="G27">
+      <c r="G28">
         <f t="shared" si="8"/>
         <v>10</v>
       </c>
-      <c r="H27">
+      <c r="H28">
         <f t="shared" si="8"/>
         <v>10</v>
       </c>
-      <c r="I27">
-        <f t="shared" ref="I27:O27" si="30">H27</f>
+      <c r="I28">
+        <f t="shared" ref="I28:O28" si="30">H28</f>
         <v>10</v>
       </c>
-      <c r="J27">
+      <c r="J28">
         <f t="shared" si="30"/>
         <v>10</v>
       </c>
-      <c r="K27">
+      <c r="K28">
         <f t="shared" si="30"/>
         <v>10</v>
       </c>
-      <c r="L27">
+      <c r="L28">
         <f t="shared" si="30"/>
         <v>10</v>
       </c>
-      <c r="M27">
+      <c r="M28">
         <f t="shared" si="30"/>
         <v>10</v>
       </c>
-      <c r="N27">
+      <c r="N28">
         <f t="shared" si="30"/>
         <v>10</v>
       </c>
-      <c r="O27">
+      <c r="O28">
         <f t="shared" si="30"/>
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A28" s="8"/>
-      <c r="B28" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="E28">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="F28">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="G28">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="H28">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="I28">
-        <f t="shared" ref="I28:O28" si="31">H28</f>
-        <v>0</v>
-      </c>
-      <c r="J28">
-        <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-      <c r="K28">
-        <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-      <c r="L28">
-        <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-      <c r="M28">
-        <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-      <c r="N28">
-        <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-      <c r="O28">
-        <f t="shared" si="31"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="8"/>
       <c r="B29" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -2242,555 +2194,555 @@
         <v>0</v>
       </c>
       <c r="I29">
-        <f t="shared" ref="I29:O29" si="32">H29</f>
+        <f t="shared" ref="I29:O29" si="31">H29</f>
         <v>0</v>
       </c>
       <c r="J29">
-        <f t="shared" si="32"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="K29">
-        <f t="shared" si="32"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="L29">
-        <f t="shared" si="32"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="M29">
-        <f t="shared" si="32"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="N29">
-        <f t="shared" si="32"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="O29">
-        <f t="shared" si="32"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="31"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="8"/>
       <c r="B30" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <f t="shared" ref="I30:O30" si="32">H30</f>
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="L30">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="M30">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="N30">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <f t="shared" si="32"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" s="8"/>
+      <c r="B31" t="s">
         <v>28</v>
       </c>
-      <c r="C30">
+      <c r="C31">
         <v>14</v>
       </c>
-      <c r="D30">
+      <c r="D31">
         <f t="shared" si="8"/>
         <v>14</v>
       </c>
-      <c r="E30">
+      <c r="E31">
         <f t="shared" si="8"/>
         <v>14</v>
       </c>
-      <c r="F30">
+      <c r="F31">
         <f t="shared" si="8"/>
         <v>14</v>
       </c>
-      <c r="G30">
+      <c r="G31">
         <f t="shared" si="8"/>
         <v>14</v>
       </c>
-      <c r="H30">
+      <c r="H31">
         <f t="shared" si="8"/>
         <v>14</v>
       </c>
-      <c r="I30">
-        <f t="shared" ref="I30:O30" si="33">H30</f>
+      <c r="I31">
+        <f t="shared" ref="I31:O31" si="33">H31</f>
         <v>14</v>
       </c>
-      <c r="J30">
+      <c r="J31">
         <f t="shared" si="33"/>
         <v>14</v>
       </c>
-      <c r="K30">
+      <c r="K31">
         <f t="shared" si="33"/>
         <v>14</v>
       </c>
-      <c r="L30">
+      <c r="L31">
         <f t="shared" si="33"/>
         <v>14</v>
       </c>
-      <c r="M30">
+      <c r="M31">
         <f t="shared" si="33"/>
         <v>14</v>
       </c>
-      <c r="N30">
+      <c r="N31">
         <f t="shared" si="33"/>
         <v>14</v>
       </c>
-      <c r="O30">
+      <c r="O31">
         <f t="shared" si="33"/>
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A31" s="8"/>
-      <c r="B31" t="s">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" s="8"/>
+      <c r="B32" t="s">
         <v>29</v>
       </c>
-      <c r="C31" s="4">
+      <c r="C32" s="4">
         <v>45026</v>
       </c>
-      <c r="D31" s="4">
+      <c r="D32" s="4">
         <f t="shared" si="8"/>
         <v>45026</v>
       </c>
-      <c r="E31" s="4">
+      <c r="E32" s="4">
         <f t="shared" si="8"/>
         <v>45026</v>
       </c>
-      <c r="F31" s="4">
+      <c r="F32" s="4">
         <f t="shared" si="8"/>
         <v>45026</v>
       </c>
-      <c r="G31" s="4">
+      <c r="G32" s="4">
         <f t="shared" si="8"/>
         <v>45026</v>
       </c>
-      <c r="H31" s="4">
+      <c r="H32" s="4">
         <f t="shared" si="8"/>
         <v>45026</v>
       </c>
-      <c r="I31" s="4">
-        <f t="shared" ref="I31:O31" si="34">H31</f>
+      <c r="I32" s="4">
+        <f t="shared" ref="I32:O32" si="34">H32</f>
         <v>45026</v>
       </c>
-      <c r="J31" s="4">
+      <c r="J32" s="4">
         <f t="shared" si="34"/>
         <v>45026</v>
       </c>
-      <c r="K31" s="4">
+      <c r="K32" s="4">
         <f t="shared" si="34"/>
         <v>45026</v>
       </c>
-      <c r="L31" s="4">
+      <c r="L32" s="4">
         <f t="shared" si="34"/>
         <v>45026</v>
       </c>
-      <c r="M31" s="4">
+      <c r="M32" s="4">
         <f t="shared" si="34"/>
         <v>45026</v>
       </c>
-      <c r="N31" s="4">
+      <c r="N32" s="4">
         <f t="shared" si="34"/>
         <v>45026</v>
       </c>
-      <c r="O31" s="4">
+      <c r="O32" s="4">
         <f t="shared" si="34"/>
         <v>45026</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A32" s="8"/>
-      <c r="B32" t="s">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" s="8"/>
+      <c r="B33" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="6" t="str">
+      <c r="C33" s="6" t="str">
         <f>C2</f>
         <v>Seed</v>
       </c>
-      <c r="D32" s="6" t="str">
-        <f t="shared" ref="D32:H32" si="35">D2</f>
+      <c r="D33" s="6" t="str">
+        <f t="shared" ref="D33:H33" si="35">D2</f>
         <v>Seed</v>
       </c>
-      <c r="E32" s="6" t="str">
+      <c r="E33" s="6" t="str">
         <f t="shared" si="35"/>
         <v>Seed</v>
       </c>
-      <c r="F32" s="6" t="str">
+      <c r="F33" s="6" t="str">
         <f t="shared" si="35"/>
         <v>Seed</v>
       </c>
-      <c r="G32" s="6" t="str">
+      <c r="G33" s="6" t="str">
         <f t="shared" si="35"/>
         <v>Seed</v>
       </c>
-      <c r="H32" s="6" t="str">
+      <c r="H33" s="6" t="str">
         <f t="shared" si="35"/>
         <v>Seed</v>
       </c>
-      <c r="I32" s="6" t="str">
-        <f t="shared" ref="I32:N32" si="36">I2</f>
+      <c r="I33" s="6" t="str">
+        <f t="shared" ref="I33:N33" si="36">I2</f>
         <v>Seedling</v>
       </c>
-      <c r="J32" s="6" t="str">
+      <c r="J33" s="6" t="str">
         <f t="shared" si="36"/>
         <v>Seedling</v>
       </c>
-      <c r="K32" s="6" t="str">
+      <c r="K33" s="6" t="str">
         <f t="shared" si="36"/>
         <v>Seedling</v>
       </c>
-      <c r="L32" s="6" t="str">
+      <c r="L33" s="6" t="str">
         <f t="shared" si="36"/>
         <v>Seedling</v>
       </c>
-      <c r="M32" s="6" t="str">
+      <c r="M33" s="6" t="str">
         <f t="shared" si="36"/>
         <v>Seedling</v>
       </c>
-      <c r="N32" s="6" t="str">
+      <c r="N33" s="6" t="str">
         <f t="shared" si="36"/>
         <v>Seedling</v>
       </c>
-      <c r="O32" s="6" t="str">
-        <f t="shared" ref="O32" si="37">O2</f>
+      <c r="O33" s="6" t="str">
+        <f t="shared" ref="O33" si="37">O2</f>
         <v>Seedling</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A33" s="8"/>
-      <c r="B33" t="s">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" s="8"/>
+      <c r="B34" t="s">
         <v>31</v>
       </c>
-      <c r="C33" s="4">
+      <c r="C34" s="4">
         <v>45326</v>
       </c>
-      <c r="D33" s="4">
+      <c r="D34" s="4">
         <f t="shared" si="8"/>
         <v>45326</v>
       </c>
-      <c r="E33" s="4">
+      <c r="E34" s="4">
         <f t="shared" si="8"/>
         <v>45326</v>
       </c>
-      <c r="F33" s="4">
+      <c r="F34" s="4">
         <f t="shared" si="8"/>
         <v>45326</v>
       </c>
-      <c r="G33" s="4">
+      <c r="G34" s="4">
         <f t="shared" si="8"/>
         <v>45326</v>
       </c>
-      <c r="H33" s="4">
+      <c r="H34" s="4">
         <f t="shared" si="8"/>
         <v>45326</v>
       </c>
-      <c r="I33" s="4">
-        <f t="shared" ref="I33:O33" si="38">H33</f>
+      <c r="I34" s="4">
+        <f t="shared" ref="I34:O34" si="38">H34</f>
         <v>45326</v>
       </c>
-      <c r="J33" s="4">
+      <c r="J34" s="4">
         <f t="shared" si="38"/>
         <v>45326</v>
       </c>
-      <c r="K33" s="4">
+      <c r="K34" s="4">
         <f t="shared" si="38"/>
         <v>45326</v>
       </c>
-      <c r="L33" s="4">
+      <c r="L34" s="4">
         <f t="shared" si="38"/>
         <v>45326</v>
       </c>
-      <c r="M33" s="4">
+      <c r="M34" s="4">
         <f t="shared" si="38"/>
         <v>45326</v>
       </c>
-      <c r="N33" s="4">
+      <c r="N34" s="4">
         <f t="shared" si="38"/>
         <v>45326</v>
       </c>
-      <c r="O33" s="4">
+      <c r="O34" s="4">
         <f t="shared" si="38"/>
         <v>45326</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A34" s="8"/>
-      <c r="B34" t="s">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" s="8"/>
+      <c r="B35" t="s">
         <v>32</v>
       </c>
-      <c r="C34" s="6" t="str">
-        <f t="shared" ref="C34:H34" si="39">C1</f>
+      <c r="C35" s="6" t="str">
+        <f t="shared" ref="C35:H35" si="39">C1</f>
         <v>Vegetative</v>
       </c>
-      <c r="D34" s="6" t="str">
+      <c r="D35" s="6" t="str">
         <f t="shared" si="39"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="E34" s="6" t="str">
+      <c r="E35" s="6" t="str">
         <f t="shared" si="39"/>
         <v>MidReproductive</v>
       </c>
-      <c r="F34" s="6" t="str">
+      <c r="F35" s="6" t="str">
         <f t="shared" si="39"/>
         <v>LateReproductive</v>
       </c>
-      <c r="G34" s="6" t="str">
+      <c r="G35" s="6" t="str">
         <f t="shared" si="39"/>
         <v>Maturity</v>
       </c>
-      <c r="H34" s="6" t="str">
+      <c r="H35" s="6" t="str">
         <f t="shared" si="39"/>
         <v>Late</v>
       </c>
-      <c r="I34" s="6" t="str">
-        <f t="shared" ref="I34:N34" si="40">I1</f>
+      <c r="I35" s="6" t="str">
+        <f t="shared" ref="I35:N35" si="40">I1</f>
         <v>Vegetative</v>
       </c>
-      <c r="J34" s="6" t="str">
+      <c r="J35" s="6" t="str">
         <f t="shared" si="40"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="K34" s="6" t="str">
+      <c r="K35" s="6" t="str">
         <f t="shared" si="40"/>
         <v>MidReproductive</v>
       </c>
-      <c r="L34" s="6" t="str">
+      <c r="L35" s="6" t="str">
         <f t="shared" si="40"/>
         <v>LateReproductive</v>
       </c>
-      <c r="M34" s="6" t="str">
+      <c r="M35" s="6" t="str">
         <f t="shared" si="40"/>
         <v>Maturity</v>
       </c>
-      <c r="N34" s="6" t="str">
+      <c r="N35" s="6" t="str">
         <f t="shared" si="40"/>
         <v>Late</v>
       </c>
-      <c r="O34" s="6" t="str">
-        <f t="shared" ref="O34" si="41">O1</f>
+      <c r="O35" s="6" t="str">
+        <f t="shared" ref="O35" si="41">O1</f>
         <v>Maturity</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="8"/>
-      <c r="B35" t="s">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" s="8"/>
+      <c r="B36" t="s">
         <v>33</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C36" t="s">
         <v>22</v>
       </c>
-      <c r="D35" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="E35" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="F35" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="G35" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="H35" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="I35" t="str">
-        <f t="shared" ref="I35:O35" si="42">H35</f>
-        <v>None removed</v>
-      </c>
-      <c r="J35" t="str">
+      <c r="D36" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="E36" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="F36" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="G36" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="H36" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="I36" t="str">
+        <f t="shared" ref="I36:O36" si="42">H36</f>
+        <v>None removed</v>
+      </c>
+      <c r="J36" t="str">
         <f t="shared" si="42"/>
         <v>None removed</v>
       </c>
-      <c r="K35" t="str">
+      <c r="K36" t="str">
         <f t="shared" si="42"/>
         <v>None removed</v>
       </c>
-      <c r="L35" t="str">
+      <c r="L36" t="str">
         <f t="shared" si="42"/>
         <v>None removed</v>
       </c>
-      <c r="M35" t="str">
+      <c r="M36" t="str">
         <f t="shared" si="42"/>
         <v>None removed</v>
       </c>
-      <c r="N35" t="str">
+      <c r="N36" t="str">
         <f t="shared" si="42"/>
         <v>None removed</v>
       </c>
-      <c r="O35" t="str">
+      <c r="O36" t="str">
         <f t="shared" si="42"/>
         <v>None removed</v>
       </c>
     </row>
-    <row r="36" spans="1:15" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="8"/>
-      <c r="B36" s="1" t="s">
+    <row r="37" spans="1:15" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="8"/>
+      <c r="B37" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C37" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D36" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="E36" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="F36" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="G36" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="H36" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="I36" s="1" t="str">
-        <f t="shared" ref="I36:O36" si="43">H36</f>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="J36" s="1" t="str">
+      <c r="D37" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="E37" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="F37" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="G37" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="H37" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="I37" s="1" t="str">
+        <f t="shared" ref="I37:O37" si="43">H37</f>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="J37" s="1" t="str">
         <f t="shared" si="43"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="K36" s="1" t="str">
+      <c r="K37" s="1" t="str">
         <f t="shared" si="43"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="L36" s="1" t="str">
+      <c r="L37" s="1" t="str">
         <f t="shared" si="43"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="M36" s="1" t="str">
+      <c r="M37" s="1" t="str">
         <f t="shared" si="43"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="N36" s="1" t="str">
+      <c r="N37" s="1" t="str">
         <f t="shared" si="43"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="O36" s="1" t="str">
+      <c r="O37" s="1" t="str">
         <f t="shared" si="43"/>
         <v>Full (Plough)</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A37" s="9" t="s">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A38" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B38" t="s">
         <v>35</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C38" t="s">
         <v>36</v>
       </c>
-      <c r="D37" t="str">
+      <c r="D38" t="str">
         <f t="shared" si="8"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="E37" t="str">
+      <c r="E38" t="str">
         <f t="shared" si="8"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="F37" t="str">
+      <c r="F38" t="str">
         <f t="shared" si="8"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="G37" t="str">
+      <c r="G38" t="str">
         <f t="shared" si="8"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="H37" t="str">
+      <c r="H38" t="str">
         <f t="shared" si="8"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="I37" t="str">
-        <f t="shared" ref="I37:O37" si="44">H37</f>
+      <c r="I38" t="str">
+        <f t="shared" ref="I38:O38" si="44">H38</f>
         <v>Oat Fodder General</v>
       </c>
-      <c r="J37" t="str">
+      <c r="J38" t="str">
         <f t="shared" si="44"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="K37" t="str">
+      <c r="K38" t="str">
         <f t="shared" si="44"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="L37" t="str">
+      <c r="L38" t="str">
         <f t="shared" si="44"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="M37" t="str">
+      <c r="M38" t="str">
         <f t="shared" si="44"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="N37" t="str">
+      <c r="N38" t="str">
         <f t="shared" si="44"/>
         <v>Oat Fodder General</v>
       </c>
-      <c r="O37" t="str">
+      <c r="O38" t="str">
         <f t="shared" si="44"/>
         <v>Oat Fodder General</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="9"/>
-      <c r="B38" t="s">
-        <v>55</v>
-      </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
-      <c r="D38">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="E38">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="F38">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="G38">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="H38">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="I38">
-        <f t="shared" ref="I38:O38" si="45">H38</f>
-        <v>0</v>
-      </c>
-      <c r="J38">
-        <f t="shared" si="45"/>
-        <v>0</v>
-      </c>
-      <c r="K38">
-        <f t="shared" si="45"/>
-        <v>0</v>
-      </c>
-      <c r="L38">
-        <f t="shared" si="45"/>
-        <v>0</v>
-      </c>
-      <c r="M38">
-        <f t="shared" si="45"/>
-        <v>0</v>
-      </c>
-      <c r="N38">
-        <f t="shared" si="45"/>
-        <v>0</v>
-      </c>
-      <c r="O38">
-        <f t="shared" si="45"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
       <c r="B39" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -2816,38 +2768,38 @@
         <v>0</v>
       </c>
       <c r="I39">
-        <f t="shared" ref="I39:O39" si="46">H39</f>
+        <f t="shared" ref="I39:O39" si="45">H39</f>
         <v>0</v>
       </c>
       <c r="J39">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="K39">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="L39">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="M39">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="N39">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="O39">
-        <f t="shared" si="46"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
       <c r="B40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -2873,38 +2825,38 @@
         <v>0</v>
       </c>
       <c r="I40">
-        <f t="shared" ref="I40:O40" si="47">H40</f>
+        <f t="shared" ref="I40:O40" si="46">H40</f>
         <v>0</v>
       </c>
       <c r="J40">
-        <f t="shared" si="47"/>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="K40">
-        <f t="shared" si="47"/>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="L40">
-        <f t="shared" si="47"/>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="M40">
-        <f t="shared" si="47"/>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="N40">
-        <f t="shared" si="47"/>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="O40">
-        <f t="shared" si="47"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="9"/>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41">
         <v>0</v>
@@ -2930,382 +2882,439 @@
         <v>0</v>
       </c>
       <c r="I41">
-        <f t="shared" ref="I41:O41" si="48">H41</f>
+        <f t="shared" ref="I41:O41" si="47">H41</f>
         <v>0</v>
       </c>
       <c r="J41">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="K41">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="L41">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="M41">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="N41">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="O41">
-        <f t="shared" si="48"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+        <f t="shared" si="47"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
       <c r="B42" t="s">
+        <v>39</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <f t="shared" ref="I42:O42" si="48">H42</f>
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="K42">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="L42">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="M42">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="N42">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="O42">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="9"/>
+      <c r="B43" t="s">
         <v>40</v>
       </c>
-      <c r="C42" s="4">
+      <c r="C43" s="4">
         <v>45355</v>
       </c>
-      <c r="D42" s="4">
+      <c r="D43" s="4">
         <f t="shared" si="8"/>
         <v>45355</v>
       </c>
-      <c r="E42" s="4">
+      <c r="E43" s="4">
         <f t="shared" si="8"/>
         <v>45355</v>
       </c>
-      <c r="F42" s="4">
+      <c r="F43" s="4">
         <f t="shared" si="8"/>
         <v>45355</v>
       </c>
-      <c r="G42" s="4">
+      <c r="G43" s="4">
         <f t="shared" si="8"/>
         <v>45355</v>
       </c>
-      <c r="H42" s="4">
+      <c r="H43" s="4">
         <f t="shared" si="8"/>
         <v>45355</v>
       </c>
-      <c r="I42" s="4">
-        <f t="shared" ref="I42:O42" si="49">H42</f>
+      <c r="I43" s="4">
+        <f t="shared" ref="I43:O43" si="49">H43</f>
         <v>45355</v>
       </c>
-      <c r="J42" s="4">
+      <c r="J43" s="4">
         <f t="shared" si="49"/>
         <v>45355</v>
       </c>
-      <c r="K42" s="4">
+      <c r="K43" s="4">
         <f t="shared" si="49"/>
         <v>45355</v>
       </c>
-      <c r="L42" s="4">
+      <c r="L43" s="4">
         <f t="shared" si="49"/>
         <v>45355</v>
       </c>
-      <c r="M42" s="4">
+      <c r="M43" s="4">
         <f t="shared" si="49"/>
         <v>45355</v>
       </c>
-      <c r="N42" s="4">
+      <c r="N43" s="4">
         <f t="shared" si="49"/>
         <v>45355</v>
       </c>
-      <c r="O42" s="4">
+      <c r="O43" s="4">
         <f t="shared" si="49"/>
         <v>45355</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A43" s="9"/>
-      <c r="B43" t="s">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="9"/>
+      <c r="B44" t="s">
         <v>41</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C44" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D43" s="3" t="str">
+      <c r="D44" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="E43" s="3" t="str">
+      <c r="E44" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="F43" s="3" t="str">
+      <c r="F44" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="G43" s="3" t="str">
+      <c r="G44" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="H43" s="3" t="str">
+      <c r="H44" s="3" t="str">
         <f t="shared" si="8"/>
         <v>Seed</v>
       </c>
-      <c r="I43" s="3" t="str">
-        <f t="shared" ref="I43:O43" si="50">H43</f>
+      <c r="I44" s="3" t="str">
+        <f t="shared" ref="I44:O44" si="50">H44</f>
         <v>Seed</v>
       </c>
-      <c r="J43" s="3" t="str">
+      <c r="J44" s="3" t="str">
         <f t="shared" si="50"/>
         <v>Seed</v>
       </c>
-      <c r="K43" s="3" t="str">
+      <c r="K44" s="3" t="str">
         <f t="shared" si="50"/>
         <v>Seed</v>
       </c>
-      <c r="L43" s="3" t="str">
+      <c r="L44" s="3" t="str">
         <f t="shared" si="50"/>
         <v>Seed</v>
       </c>
-      <c r="M43" s="3" t="str">
+      <c r="M44" s="3" t="str">
         <f t="shared" si="50"/>
         <v>Seed</v>
       </c>
-      <c r="N43" s="3" t="str">
+      <c r="N44" s="3" t="str">
         <f t="shared" si="50"/>
         <v>Seed</v>
       </c>
-      <c r="O43" s="3" t="str">
+      <c r="O44" s="3" t="str">
         <f t="shared" si="50"/>
         <v>Seed</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A44" s="9"/>
-      <c r="B44" t="s">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A45" s="9"/>
+      <c r="B45" t="s">
         <v>42</v>
       </c>
-      <c r="C44" s="4">
+      <c r="C45" s="4">
         <v>45387</v>
       </c>
-      <c r="D44" s="4">
+      <c r="D45" s="4">
         <f t="shared" si="8"/>
         <v>45387</v>
       </c>
-      <c r="E44" s="4">
+      <c r="E45" s="4">
         <f t="shared" si="8"/>
         <v>45387</v>
       </c>
-      <c r="F44" s="4">
+      <c r="F45" s="4">
         <f t="shared" si="8"/>
         <v>45387</v>
       </c>
-      <c r="G44" s="4">
+      <c r="G45" s="4">
         <f t="shared" si="8"/>
         <v>45387</v>
       </c>
-      <c r="H44" s="4">
+      <c r="H45" s="4">
         <f t="shared" si="8"/>
         <v>45387</v>
       </c>
-      <c r="I44" s="4">
-        <f t="shared" ref="I44:O44" si="51">H44</f>
+      <c r="I45" s="4">
+        <f t="shared" ref="I45:O45" si="51">H45</f>
         <v>45387</v>
       </c>
-      <c r="J44" s="4">
+      <c r="J45" s="4">
         <f t="shared" si="51"/>
         <v>45387</v>
       </c>
-      <c r="K44" s="4">
+      <c r="K45" s="4">
         <f t="shared" si="51"/>
         <v>45387</v>
       </c>
-      <c r="L44" s="4">
+      <c r="L45" s="4">
         <f t="shared" si="51"/>
         <v>45387</v>
       </c>
-      <c r="M44" s="4">
+      <c r="M45" s="4">
         <f t="shared" si="51"/>
         <v>45387</v>
       </c>
-      <c r="N44" s="4">
+      <c r="N45" s="4">
         <f t="shared" si="51"/>
         <v>45387</v>
       </c>
-      <c r="O44" s="4">
+      <c r="O45" s="4">
         <f t="shared" si="51"/>
         <v>45387</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A45" s="9"/>
-      <c r="B45" t="s">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" s="9"/>
+      <c r="B46" t="s">
         <v>43</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C46" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D45" s="3" t="str">
+      <c r="D46" s="3" t="str">
         <f t="shared" si="8"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="E45" s="3" t="str">
+      <c r="E46" s="3" t="str">
         <f t="shared" si="8"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="F45" s="3" t="str">
+      <c r="F46" s="3" t="str">
         <f t="shared" si="8"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="G45" s="3" t="str">
+      <c r="G46" s="3" t="str">
         <f t="shared" si="8"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="H45" s="3" t="str">
+      <c r="H46" s="3" t="str">
         <f t="shared" si="8"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="I45" s="3" t="str">
-        <f t="shared" ref="I45:O45" si="52">H45</f>
+      <c r="I46" s="3" t="str">
+        <f t="shared" ref="I46:O46" si="52">H46</f>
         <v>EarlyReproductive</v>
       </c>
-      <c r="J45" s="3" t="str">
+      <c r="J46" s="3" t="str">
         <f t="shared" si="52"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="K45" s="3" t="str">
+      <c r="K46" s="3" t="str">
         <f t="shared" si="52"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="L45" s="3" t="str">
+      <c r="L46" s="3" t="str">
         <f t="shared" si="52"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="M45" s="3" t="str">
+      <c r="M46" s="3" t="str">
         <f t="shared" si="52"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="N45" s="3" t="str">
+      <c r="N46" s="3" t="str">
         <f t="shared" si="52"/>
         <v>EarlyReproductive</v>
       </c>
-      <c r="O45" s="3" t="str">
+      <c r="O46" s="3" t="str">
         <f t="shared" si="52"/>
         <v>EarlyReproductive</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A46" s="9"/>
-      <c r="B46" t="s">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" s="9"/>
+      <c r="B47" t="s">
         <v>45</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C47" t="s">
         <v>22</v>
       </c>
-      <c r="D46" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="E46" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="F46" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="G46" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="H46" t="str">
-        <f t="shared" si="8"/>
-        <v>None removed</v>
-      </c>
-      <c r="I46" t="str">
-        <f t="shared" ref="I46:O46" si="53">H46</f>
-        <v>None removed</v>
-      </c>
-      <c r="J46" t="str">
+      <c r="D47" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="E47" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="F47" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="G47" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="H47" t="str">
+        <f t="shared" si="8"/>
+        <v>None removed</v>
+      </c>
+      <c r="I47" t="str">
+        <f t="shared" ref="I47:O47" si="53">H47</f>
+        <v>None removed</v>
+      </c>
+      <c r="J47" t="str">
         <f t="shared" si="53"/>
         <v>None removed</v>
       </c>
-      <c r="K46" t="str">
+      <c r="K47" t="str">
         <f t="shared" si="53"/>
         <v>None removed</v>
       </c>
-      <c r="L46" t="str">
+      <c r="L47" t="str">
         <f t="shared" si="53"/>
         <v>None removed</v>
       </c>
-      <c r="M46" t="str">
+      <c r="M47" t="str">
         <f t="shared" si="53"/>
         <v>None removed</v>
       </c>
-      <c r="N46" t="str">
+      <c r="N47" t="str">
         <f t="shared" si="53"/>
         <v>None removed</v>
       </c>
-      <c r="O46" t="str">
+      <c r="O47" t="str">
         <f t="shared" si="53"/>
         <v>None removed</v>
       </c>
     </row>
-    <row r="47" spans="1:15" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="10"/>
-      <c r="B47" s="1" t="s">
+    <row r="48" spans="1:15" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="10"/>
+      <c r="B48" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C48" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D47" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="E47" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="F47" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="G47" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="H47" s="1" t="str">
-        <f t="shared" si="8"/>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="I47" s="1" t="str">
-        <f t="shared" ref="I47:O47" si="54">H47</f>
-        <v>Full (Plough)</v>
-      </c>
-      <c r="J47" s="1" t="str">
+      <c r="D48" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="E48" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="F48" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="G48" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="H48" s="1" t="str">
+        <f t="shared" si="8"/>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="I48" s="1" t="str">
+        <f t="shared" ref="I48:O48" si="54">H48</f>
+        <v>Full (Plough)</v>
+      </c>
+      <c r="J48" s="1" t="str">
         <f t="shared" si="54"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="K47" s="1" t="str">
+      <c r="K48" s="1" t="str">
         <f t="shared" si="54"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="L47" s="1" t="str">
+      <c r="L48" s="1" t="str">
         <f t="shared" si="54"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="M47" s="1" t="str">
+      <c r="M48" s="1" t="str">
         <f t="shared" si="54"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="N47" s="1" t="str">
+      <c r="N48" s="1" t="str">
         <f t="shared" si="54"/>
         <v>Full (Plough)</v>
       </c>
-      <c r="O47" s="1" t="str">
+      <c r="O48" s="1" t="str">
         <f t="shared" si="54"/>
         <v>Full (Plough)</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="A15:A25"/>
-    <mergeCell ref="A26:A36"/>
-    <mergeCell ref="A37:A47"/>
+    <mergeCell ref="A9:A15"/>
+    <mergeCell ref="A16:A26"/>
+    <mergeCell ref="A27:A37"/>
+    <mergeCell ref="A38:A48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>